<commit_message>
📊 Horarios actualizados Línea 141 - 4787
</commit_message>
<xml_diff>
--- a/data/horarios-141-2026-08-27.xlsx
+++ b/data/horarios-141-2026-08-27.xlsx
@@ -419,7 +419,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E62"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -432,14 +432,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:36:12</t>
+          <t>Última actualización: 17:43:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 26</t>
+          <t>Total filas: 57</t>
         </is>
       </c>
     </row>
@@ -1115,6 +1115,781 @@
         <v>105</v>
       </c>
       <c r="E31" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>17:47</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D32" t="n">
+        <v>4</v>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>17:48</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D33" t="n">
+        <v>5</v>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>17:50</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D34" t="n">
+        <v>7</v>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>17:52</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D35" t="n">
+        <v>9</v>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>17:56</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>16_P MOR-167 Y 521</t>
+        </is>
+      </c>
+      <c r="D36" t="n">
+        <v>13</v>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>18:01</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D37" t="n">
+        <v>18</v>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>18:02</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>16_SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D38" t="n">
+        <v>19</v>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>18:06</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>83_ALUAR</t>
+        </is>
+      </c>
+      <c r="D39" t="n">
+        <v>23</v>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>18:16</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D40" t="n">
+        <v>33</v>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>18:17</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>23_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>34</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>18:21</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D42" t="n">
+        <v>38</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>18:23</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>40</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>18:24</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D44" t="n">
+        <v>41</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D45" t="n">
+        <v>47</v>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>18:31</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>11_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D46" t="n">
+        <v>48</v>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>18:32</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D47" t="n">
+        <v>49</v>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>18:37</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D48" t="n">
+        <v>54</v>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>18:40</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>26_155 Y 38-B MALVINAS</t>
+        </is>
+      </c>
+      <c r="D49" t="n">
+        <v>57</v>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D50" t="n">
+        <v>59</v>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D51" t="n">
+        <v>63</v>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D52" t="n">
+        <v>66</v>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>18:55</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D53" t="n">
+        <v>72</v>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>19:05</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>14_ABASTO</t>
+        </is>
+      </c>
+      <c r="D54" t="n">
+        <v>82</v>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>19:06</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>15_ABASTO</t>
+        </is>
+      </c>
+      <c r="D55" t="n">
+        <v>83</v>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>19:07</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>16_P MOR-SANTA ANA</t>
+        </is>
+      </c>
+      <c r="D56" t="n">
+        <v>84</v>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>19:15</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>10_OLMOS</t>
+        </is>
+      </c>
+      <c r="D57" t="n">
+        <v>92</v>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>27_EL RETIRO</t>
+        </is>
+      </c>
+      <c r="D58" t="n">
+        <v>95</v>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>95</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>19:21</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>26_HERNANDEZ</t>
+        </is>
+      </c>
+      <c r="D60" t="n">
+        <v>98</v>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>19:30</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>17_ROMERO</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>107</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>19:39</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>11X44_ETCHEVERRY</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>116</v>
+      </c>
+      <c r="E62" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1131,7 +1906,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1144,14 +1919,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:36:12</t>
+          <t>Última actualización: 17:43:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 4</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1277,6 +2052,106 @@
         <v>103</v>
       </c>
       <c r="E9" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>59</v>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>18:46</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215B_EL PATO</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>63</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>18:49</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215A_EL PATO</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>66</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>LP1912</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>19:18</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215C_EL PATO</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>95</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>LP1912</t>
         </is>
@@ -1293,7 +2168,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1306,14 +2181,14 @@
     <row r="2">
       <c r="A2" s="1" t="inlineStr">
         <is>
-          <t>Última actualización: 07:36:12</t>
+          <t>Última actualización: 17:43:15</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="inlineStr">
         <is>
-          <t>Total filas: 5</t>
+          <t>Total filas: 8</t>
         </is>
       </c>
     </row>
@@ -1464,6 +2339,81 @@
         <v>81</v>
       </c>
       <c r="E10" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>18:42</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>215C_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D11" t="n">
+        <v>59</v>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>L6203</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>18:50</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>215B_LP-P MOR-1 Y 57</t>
+        </is>
+      </c>
+      <c r="D12" t="n">
+        <v>67</v>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6173</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>17:43:15</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>18:54</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>215A_LA PLATA</t>
+        </is>
+      </c>
+      <c r="D13" t="n">
+        <v>71</v>
+      </c>
+      <c r="E13" t="inlineStr">
         <is>
           <t>L6173</t>
         </is>

</xml_diff>